<commit_message>
ANS-006-168 - Ajout causes de décès, mobilité et période scolaire (#433)
* add observation

* update PeriodeScolaire

* update observation

* ajout Observations, mapping, exmeples

* update

* update

* update Periodescolaire

* update component

* update observation

* update PR

* update display

* update mapping

* update mapping bfcda230717d502849e364b2f7ef5644c4736c38
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-careplan-projet-personnalise.xlsx
+++ b/main/ig/StructureDefinition-tddui-careplan-projet-personnalise.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-25T14:12:38+00:00</t>
+    <t>2026-02-26T10:50:19+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1012,7 +1012,7 @@
     <t>TDDUI Status Author</t>
   </si>
   <si>
-    <t>Extension permettant de représenter la profession du professionnel.</t>
+    <t>Extension permettant de représenter l'auteur du statut.</t>
   </si>
   <si>
     <t>statutProjetPersonnalise.auteur</t>

</xml_diff>